<commit_message>
add ep5 and switch format
</commit_message>
<xml_diff>
--- a/src/data/episodes/3.xlsx
+++ b/src/data/episodes/3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>الحلقة</t>
   </si>
@@ -49,6 +49,12 @@
     <t>تعاريف</t>
   </si>
   <si>
+    <t>12:20</t>
+  </si>
+  <si>
+    <t>زوج في العربية</t>
+  </si>
+  <si>
     <t>احكام</t>
   </si>
   <si>
@@ -61,10 +67,10 @@
     <t>مواضيع</t>
   </si>
   <si>
-    <t>12:20</t>
-  </si>
-  <si>
-    <t>زوج في العربية</t>
+    <t>46:00</t>
+  </si>
+  <si>
+    <t>تاخير البيان</t>
   </si>
 </sst>
 </file>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -156,6 +162,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -500,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17.714285714285715" customWidth="1"/>
@@ -584,57 +593,59 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="B8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="6"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>15</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="8"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
+      <c r="A11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="8"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
@@ -645,10 +656,18 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C10:C11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>